<commit_message>
download all data from jatim
</commit_message>
<xml_diff>
--- a/downloads/komposisi_data/Data_Komposisi_Jenis_Sampah_SIPSN_KLHK_Jawa Timur_2024.xlsx
+++ b/downloads/komposisi_data/Data_Komposisi_Jenis_Sampah_SIPSN_KLHK_Jawa Timur_2024.xlsx
@@ -646,6 +646,1113 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B13">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C13">
+        <is>
+          <t xml:space="preserve">Kab. Bondowoso</t>
+        </is>
+      </c>
+      <c r="D13" s="66">
+        <v>33.04</v>
+      </c>
+      <c r="E13" s="66">
+        <v>13.15</v>
+      </c>
+      <c r="F13" s="66">
+        <v>15.56</v>
+      </c>
+      <c r="G13" s="66">
+        <v>20.71</v>
+      </c>
+      <c r="H13" s="66">
+        <v>0.30</v>
+      </c>
+      <c r="I13" s="66">
+        <v>1.50</v>
+      </c>
+      <c r="J13" s="66">
+        <v>0.90</v>
+      </c>
+      <c r="K13" s="66">
+        <v>0.90</v>
+      </c>
+      <c r="L13" s="66">
+        <v>13.94</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B14">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C14">
+        <is>
+          <t xml:space="preserve">Kab. Situbondo</t>
+        </is>
+      </c>
+      <c r="D14" s="66">
+        <v>41.20</v>
+      </c>
+      <c r="E14" s="66">
+        <v>15.70</v>
+      </c>
+      <c r="F14" s="66">
+        <v>17.30</v>
+      </c>
+      <c r="G14" s="66">
+        <v>23.90</v>
+      </c>
+      <c r="H14" s="66">
+        <v>0.80</v>
+      </c>
+      <c r="I14" s="66">
+        <v>0.40</v>
+      </c>
+      <c r="J14" s="66">
+        <v>0.10</v>
+      </c>
+      <c r="K14" s="66">
+        <v>0.20</v>
+      </c>
+      <c r="L14" s="66">
+        <v>0.40</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B15">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C15">
+        <is>
+          <t xml:space="preserve">Kab. Probolinggo</t>
+        </is>
+      </c>
+      <c r="D15" s="66">
+        <v>40.02</v>
+      </c>
+      <c r="E15" s="66">
+        <v>12.25</v>
+      </c>
+      <c r="F15" s="66">
+        <v>15.40</v>
+      </c>
+      <c r="G15" s="66">
+        <v>17.21</v>
+      </c>
+      <c r="H15" s="66">
+        <v>0.45</v>
+      </c>
+      <c r="I15" s="66">
+        <v>5.15</v>
+      </c>
+      <c r="J15" s="66">
+        <v>1.77</v>
+      </c>
+      <c r="K15" s="66">
+        <v>2.08</v>
+      </c>
+      <c r="L15" s="66">
+        <v>5.67</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B16">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C16">
+        <is>
+          <t xml:space="preserve">Kab. Pasuruan</t>
+        </is>
+      </c>
+      <c r="D16" s="66">
+        <v>58.50</v>
+      </c>
+      <c r="E16" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="F16" s="66">
+        <v>5.70</v>
+      </c>
+      <c r="G16" s="66">
+        <v>10.00</v>
+      </c>
+      <c r="H16" s="66">
+        <v>1.30</v>
+      </c>
+      <c r="I16" s="66">
+        <v>0.50</v>
+      </c>
+      <c r="J16" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="K16" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="L16" s="66">
+        <v>21.00</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B17">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C17">
+        <is>
+          <t xml:space="preserve">Kab. Sidoarjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B18">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C18">
+        <is>
+          <t xml:space="preserve">Kab. Mojokerto</t>
+        </is>
+      </c>
+      <c r="D18" s="66">
+        <v>47.88</v>
+      </c>
+      <c r="E18" s="66">
+        <v>1.91</v>
+      </c>
+      <c r="F18" s="66">
+        <v>19.54</v>
+      </c>
+      <c r="G18" s="66">
+        <v>21.07</v>
+      </c>
+      <c r="H18" s="66">
+        <v>0.53</v>
+      </c>
+      <c r="I18" s="66">
+        <v>0.47</v>
+      </c>
+      <c r="J18" s="66">
+        <v>0.17</v>
+      </c>
+      <c r="K18" s="66">
+        <v>0.24</v>
+      </c>
+      <c r="L18" s="66">
+        <v>8.19</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B19">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C19">
+        <is>
+          <t xml:space="preserve">Kab. Jombang</t>
+        </is>
+      </c>
+      <c r="D19" s="66">
+        <v>49.00</v>
+      </c>
+      <c r="E19" s="66">
+        <v>12.00</v>
+      </c>
+      <c r="F19" s="66">
+        <v>8.00</v>
+      </c>
+      <c r="G19" s="66">
+        <v>15.00</v>
+      </c>
+      <c r="H19" s="66">
+        <v>1.80</v>
+      </c>
+      <c r="I19" s="66">
+        <v>5.00</v>
+      </c>
+      <c r="J19" s="66">
+        <v>1.60</v>
+      </c>
+      <c r="K19" s="66">
+        <v>1.60</v>
+      </c>
+      <c r="L19" s="66">
+        <v>6.00</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B20">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C20">
+        <is>
+          <t xml:space="preserve">Kab. Nganjuk</t>
+        </is>
+      </c>
+      <c r="D20" s="66">
+        <v>61.50</v>
+      </c>
+      <c r="E20" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="F20" s="66">
+        <v>13.10</v>
+      </c>
+      <c r="G20" s="66">
+        <v>12.30</v>
+      </c>
+      <c r="H20" s="66">
+        <v>6.00</v>
+      </c>
+      <c r="I20" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="J20" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="K20" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="L20" s="66">
+        <v>2.10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B21">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C21">
+        <is>
+          <t xml:space="preserve">Kab. Madiun</t>
+        </is>
+      </c>
+      <c r="D21" s="66">
+        <v>39.80</v>
+      </c>
+      <c r="E21" s="66">
+        <v>11.30</v>
+      </c>
+      <c r="F21" s="66">
+        <v>13.30</v>
+      </c>
+      <c r="G21" s="66">
+        <v>19.70</v>
+      </c>
+      <c r="H21" s="66">
+        <v>5.34</v>
+      </c>
+      <c r="I21" s="66">
+        <v>2.65</v>
+      </c>
+      <c r="J21" s="66">
+        <v>2.02</v>
+      </c>
+      <c r="K21" s="66">
+        <v>4.91</v>
+      </c>
+      <c r="L21" s="66">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B22">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C22">
+        <is>
+          <t xml:space="preserve">Kab. Magetan</t>
+        </is>
+      </c>
+      <c r="D22" s="66">
+        <v>36.28</v>
+      </c>
+      <c r="E22" s="66">
+        <v>25.01</v>
+      </c>
+      <c r="F22" s="66">
+        <v>8.22</v>
+      </c>
+      <c r="G22" s="66">
+        <v>14.25</v>
+      </c>
+      <c r="H22" s="66">
+        <v>0.31</v>
+      </c>
+      <c r="I22" s="66">
+        <v>1.35</v>
+      </c>
+      <c r="J22" s="66">
+        <v>2.81</v>
+      </c>
+      <c r="K22" s="66">
+        <v>3.22</v>
+      </c>
+      <c r="L22" s="66">
+        <v>8.55</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B23">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C23">
+        <is>
+          <t xml:space="preserve">Kab. Ngawi</t>
+        </is>
+      </c>
+      <c r="D23" s="66">
+        <v>59.47</v>
+      </c>
+      <c r="E23" s="66">
+        <v>6.92</v>
+      </c>
+      <c r="F23" s="66">
+        <v>11.17</v>
+      </c>
+      <c r="G23" s="66">
+        <v>10.71</v>
+      </c>
+      <c r="H23" s="66">
+        <v>1.77</v>
+      </c>
+      <c r="I23" s="66">
+        <v>0.81</v>
+      </c>
+      <c r="J23" s="66">
+        <v>1.61</v>
+      </c>
+      <c r="K23" s="66">
+        <v>1.33</v>
+      </c>
+      <c r="L23" s="66">
+        <v>6.21</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B24">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C24">
+        <is>
+          <t xml:space="preserve">Kab. Bojonegoro</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B25">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C25">
+        <is>
+          <t xml:space="preserve">Kab. Tuban</t>
+        </is>
+      </c>
+      <c r="D25" s="66">
+        <v>58.52</v>
+      </c>
+      <c r="E25" s="66">
+        <v>15.32</v>
+      </c>
+      <c r="F25" s="66">
+        <v>5.78</v>
+      </c>
+      <c r="G25" s="66">
+        <v>11.02</v>
+      </c>
+      <c r="H25" s="66">
+        <v>0.17</v>
+      </c>
+      <c r="I25" s="66">
+        <v>1.62</v>
+      </c>
+      <c r="J25" s="66">
+        <v>0.10</v>
+      </c>
+      <c r="K25" s="66">
+        <v>1.33</v>
+      </c>
+      <c r="L25" s="66">
+        <v>6.14</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B26">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C26">
+        <is>
+          <t xml:space="preserve">Kab. Lamongan</t>
+        </is>
+      </c>
+      <c r="D26" s="66">
+        <v>30.00</v>
+      </c>
+      <c r="E26" s="66">
+        <v>12.00</v>
+      </c>
+      <c r="F26" s="66">
+        <v>9.00</v>
+      </c>
+      <c r="G26" s="66">
+        <v>18.00</v>
+      </c>
+      <c r="H26" s="66">
+        <v>8.00</v>
+      </c>
+      <c r="I26" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="J26" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="K26" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="L26" s="66">
+        <v>18.00</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B27">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C27">
+        <is>
+          <t xml:space="preserve">Kab. Gresik</t>
+        </is>
+      </c>
+      <c r="D27" s="66">
+        <v>55.29</v>
+      </c>
+      <c r="E27" s="66">
+        <v>10.29</v>
+      </c>
+      <c r="F27" s="66">
+        <v>4.47</v>
+      </c>
+      <c r="G27" s="66">
+        <v>11.58</v>
+      </c>
+      <c r="H27" s="66">
+        <v>0.47</v>
+      </c>
+      <c r="I27" s="66">
+        <v>4.84</v>
+      </c>
+      <c r="J27" s="66">
+        <v>2.02</v>
+      </c>
+      <c r="K27" s="66">
+        <v>1.37</v>
+      </c>
+      <c r="L27" s="66">
+        <v>9.66</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B28">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C28">
+        <is>
+          <t xml:space="preserve">Kab. Bangkalan</t>
+        </is>
+      </c>
+      <c r="D28" s="66">
+        <v>52.32</v>
+      </c>
+      <c r="E28" s="66">
+        <v>15.32</v>
+      </c>
+      <c r="F28" s="66">
+        <v>9.72</v>
+      </c>
+      <c r="G28" s="66">
+        <v>14.97</v>
+      </c>
+      <c r="H28" s="66">
+        <v>0.43</v>
+      </c>
+      <c r="I28" s="66">
+        <v>1.02</v>
+      </c>
+      <c r="J28" s="66">
+        <v>0.29</v>
+      </c>
+      <c r="K28" s="66">
+        <v>2.93</v>
+      </c>
+      <c r="L28" s="66">
+        <v>3.00</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B29">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C29">
+        <is>
+          <t xml:space="preserve">Kab. Sampang</t>
+        </is>
+      </c>
+      <c r="D29" s="66">
+        <v>43.00</v>
+      </c>
+      <c r="E29" s="66">
+        <v>10.00</v>
+      </c>
+      <c r="F29" s="66">
+        <v>5.00</v>
+      </c>
+      <c r="G29" s="66">
+        <v>13.00</v>
+      </c>
+      <c r="H29" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="I29" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="J29" s="66">
+        <v>1.00</v>
+      </c>
+      <c r="K29" s="66">
+        <v>5.00</v>
+      </c>
+      <c r="L29" s="66">
+        <v>20.00</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B30">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C30">
+        <is>
+          <t xml:space="preserve">Kab. Pamekasan</t>
+        </is>
+      </c>
+      <c r="D30" s="66">
+        <v>55.00</v>
+      </c>
+      <c r="E30" s="66">
+        <v>4.00</v>
+      </c>
+      <c r="F30" s="66">
+        <v>7.00</v>
+      </c>
+      <c r="G30" s="66">
+        <v>13.00</v>
+      </c>
+      <c r="H30" s="66">
+        <v>3.00</v>
+      </c>
+      <c r="I30" s="66">
+        <v>5.00</v>
+      </c>
+      <c r="J30" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="K30" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="L30" s="66">
+        <v>9.00</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B31">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C31">
+        <is>
+          <t xml:space="preserve">Kab. Sumenep</t>
+        </is>
+      </c>
+      <c r="D31" s="66">
+        <v>41.92</v>
+      </c>
+      <c r="E31" s="66">
+        <v>11.34</v>
+      </c>
+      <c r="F31" s="66">
+        <v>9.89</v>
+      </c>
+      <c r="G31" s="66">
+        <v>24.77</v>
+      </c>
+      <c r="H31" s="66">
+        <v>0.89</v>
+      </c>
+      <c r="I31" s="66">
+        <v>8.04</v>
+      </c>
+      <c r="J31" s="66">
+        <v>0.74</v>
+      </c>
+      <c r="K31" s="66">
+        <v>1.15</v>
+      </c>
+      <c r="L31" s="66">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B32">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C32">
+        <is>
+          <t xml:space="preserve">Kota Kediri</t>
+        </is>
+      </c>
+      <c r="D32" s="66">
+        <v>61.20</v>
+      </c>
+      <c r="E32" s="66">
+        <v>7.00</v>
+      </c>
+      <c r="F32" s="66">
+        <v>13.50</v>
+      </c>
+      <c r="G32" s="66">
+        <v>12.60</v>
+      </c>
+      <c r="H32" s="66">
+        <v>2.50</v>
+      </c>
+      <c r="I32" s="66">
+        <v>0.70</v>
+      </c>
+      <c r="J32" s="66">
+        <v>0.50</v>
+      </c>
+      <c r="K32" s="66">
+        <v>0.50</v>
+      </c>
+      <c r="L32" s="66">
+        <v>1.50</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B33">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C33">
+        <is>
+          <t xml:space="preserve">Kota Blitar</t>
+        </is>
+      </c>
+      <c r="D33" s="66">
+        <v>42.40</v>
+      </c>
+      <c r="E33" s="66">
+        <v>13.20</v>
+      </c>
+      <c r="F33" s="66">
+        <v>8.56</v>
+      </c>
+      <c r="G33" s="66">
+        <v>16.50</v>
+      </c>
+      <c r="H33" s="66">
+        <v>3.80</v>
+      </c>
+      <c r="I33" s="66">
+        <v>2.60</v>
+      </c>
+      <c r="J33" s="66">
+        <v>2.85</v>
+      </c>
+      <c r="K33" s="66">
+        <v>2.94</v>
+      </c>
+      <c r="L33" s="66">
+        <v>7.15</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B34">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C34">
+        <is>
+          <t xml:space="preserve">Kota Malang</t>
+        </is>
+      </c>
+      <c r="D34" s="66">
+        <v>57.86</v>
+      </c>
+      <c r="E34" s="66">
+        <v>3.80</v>
+      </c>
+      <c r="F34" s="66">
+        <v>8.00</v>
+      </c>
+      <c r="G34" s="66">
+        <v>16.45</v>
+      </c>
+      <c r="H34" s="66">
+        <v>0.99</v>
+      </c>
+      <c r="I34" s="66">
+        <v>0.53</v>
+      </c>
+      <c r="J34" s="66">
+        <v>0.27</v>
+      </c>
+      <c r="K34" s="66">
+        <v>1.78</v>
+      </c>
+      <c r="L34" s="66">
+        <v>10.32</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B35">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C35">
+        <is>
+          <t xml:space="preserve">Kota Probolinggo</t>
+        </is>
+      </c>
+      <c r="D35" s="66">
+        <v>6.58</v>
+      </c>
+      <c r="E35" s="66">
+        <v>39.16</v>
+      </c>
+      <c r="F35" s="66">
+        <v>8.08</v>
+      </c>
+      <c r="G35" s="66">
+        <v>10.89</v>
+      </c>
+      <c r="H35" s="66">
+        <v>6.33</v>
+      </c>
+      <c r="I35" s="66">
+        <v>6.86</v>
+      </c>
+      <c r="J35" s="66">
+        <v>6.41</v>
+      </c>
+      <c r="K35" s="66">
+        <v>7.93</v>
+      </c>
+      <c r="L35" s="66">
+        <v>7.76</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B36">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C36">
+        <is>
+          <t xml:space="preserve">Kota Pasuruan</t>
+        </is>
+      </c>
+      <c r="D36" s="66">
+        <v>30.00</v>
+      </c>
+      <c r="E36" s="66">
+        <v>10.00</v>
+      </c>
+      <c r="F36" s="66">
+        <v>17.72</v>
+      </c>
+      <c r="G36" s="66">
+        <v>30.21</v>
+      </c>
+      <c r="H36" s="66">
+        <v>8.77</v>
+      </c>
+      <c r="I36" s="66">
+        <v>0.03</v>
+      </c>
+      <c r="J36" s="66">
+        <v>0.90</v>
+      </c>
+      <c r="K36" s="66">
+        <v>1.19</v>
+      </c>
+      <c r="L36" s="66">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B37">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C37">
+        <is>
+          <t xml:space="preserve">Kota Mojokerto</t>
+        </is>
+      </c>
+      <c r="D37" s="66">
+        <v>36.07</v>
+      </c>
+      <c r="E37" s="66">
+        <v>11.42</v>
+      </c>
+      <c r="F37" s="66">
+        <v>9.88</v>
+      </c>
+      <c r="G37" s="66">
+        <v>38.80</v>
+      </c>
+      <c r="H37" s="66">
+        <v>1.44</v>
+      </c>
+      <c r="I37" s="66">
+        <v>0.12</v>
+      </c>
+      <c r="K37" s="66">
+        <v>2.24</v>
+      </c>
+      <c r="L37" s="66">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B38">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C38">
+        <is>
+          <t xml:space="preserve">Kota Madiun</t>
+        </is>
+      </c>
+      <c r="D38" s="66">
+        <v>59.07</v>
+      </c>
+      <c r="E38" s="66">
+        <v>0.60</v>
+      </c>
+      <c r="F38" s="66">
+        <v>9.40</v>
+      </c>
+      <c r="G38" s="66">
+        <v>16.90</v>
+      </c>
+      <c r="H38" s="66">
+        <v>0.62</v>
+      </c>
+      <c r="I38" s="66">
+        <v>2.00</v>
+      </c>
+      <c r="J38" s="66">
+        <v>0.50</v>
+      </c>
+      <c r="K38" s="66">
+        <v>0.80</v>
+      </c>
+      <c r="L38" s="66">
+        <v>10.10</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B39">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C39">
+        <is>
+          <t xml:space="preserve">Kota Surabaya</t>
+        </is>
+      </c>
+      <c r="D39" s="66">
+        <v>55.48</v>
+      </c>
+      <c r="E39" s="66">
+        <v>2.25</v>
+      </c>
+      <c r="F39" s="66">
+        <v>3.05</v>
+      </c>
+      <c r="G39" s="66">
+        <v>22.01</v>
+      </c>
+      <c r="H39" s="66">
+        <v>0.25</v>
+      </c>
+      <c r="I39" s="66">
+        <v>5.75</v>
+      </c>
+      <c r="J39" s="66">
+        <v>1.35</v>
+      </c>
+      <c r="K39" s="66">
+        <v>0.50</v>
+      </c>
+      <c r="L39" s="66">
+        <v>9.36</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="65">
+        <v>2024</v>
+      </c>
+      <c t="inlineStr" r="B40">
+        <is>
+          <t xml:space="preserve">Jawa Timur</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C40">
+        <is>
+          <t xml:space="preserve">Kota Batu</t>
+        </is>
+      </c>
+      <c r="D40" s="66">
+        <v>22.00</v>
+      </c>
+      <c r="F40" s="66">
+        <v>0.45</v>
+      </c>
+      <c r="G40" s="66">
+        <v>1.01</v>
+      </c>
+      <c r="H40" s="66">
+        <v>0.00</v>
+      </c>
+      <c r="K40" s="66">
+        <v>0.07</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>

</xml_diff>